<commit_message>
Adiciona suporte para importação de arquivos XLSX e CSV na análise de margem; otimiza o tratamento de dados e a inserção no banco de dados.
</commit_message>
<xml_diff>
--- a/frontend/xlsx_models/modelo-analise-margem-sejaap.xlsx
+++ b/frontend/xlsx_models/modelo-analise-margem-sejaap.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cirog\OneDrive\Área de Trabalho\UniqCode Projetos\Modelos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cirog\OneDrive\Área de Trabalho\SejaAP-sistema\frontend\xlsx_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06FC03F9-B34C-4481-A8C1-1F567BB54420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9643A2B9-DB31-437F-9BD1-32A4206C419E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2985" yWindow="2985" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>PRODUTO OU SERVIÇO</t>
   </si>
@@ -60,23 +60,19 @@
   </si>
   <si>
     <t>FRETE</t>
+  </si>
+  <si>
+    <t>REGISTRO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -113,7 +109,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,19 +408,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
@@ -433,9 +429,12 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="M10" s="2"/>
+      <c r="M10" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>